<commit_message>
Update Test Excel File
</commit_message>
<xml_diff>
--- a/ep16-spring-transaction/online-shop-test-data.xlsx
+++ b/ep16-spring-transaction/online-shop-test-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/minlwin/git/spring-weekend-202603/ep16-spring-transaction/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8762BCBB-6A47-6C45-A908-7F123EB4B6D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38AA209C-EBCC-2849-A123-BA5EFA83BDD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="25600" windowHeight="12800" activeTab="2" xr2:uid="{B0DF375E-B9E1-2C42-A1BE-A72AC035EBB6}"/>
+    <workbookView xWindow="2320" yWindow="660" windowWidth="25600" windowHeight="12800" xr2:uid="{B0DF375E-B9E1-2C42-A1BE-A72AC035EBB6}"/>
   </bookViews>
   <sheets>
     <sheet name="CRUD" sheetId="5" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="63">
   <si>
     <t>SUPPLIER</t>
   </si>
@@ -224,6 +224,15 @@
   </si>
   <si>
     <t>quantity</t>
+  </si>
+  <si>
+    <t>thiri@example.com</t>
+  </si>
+  <si>
+    <t>nyein@example.com</t>
+  </si>
+  <si>
+    <t>shwe@example.com</t>
   </si>
 </sst>
 </file>
@@ -857,11 +866,11 @@
         <v>36</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>32</v>
+        <v>60</v>
       </c>
       <c r="E3" t="str">
         <f t="shared" ref="E3:E5" si="0">_xlfn.CONCAT("INSERT INTO supplier (", A$1, ", ",B$1, ", ",C$1, ", ",D$1, ") values (", A3, ",'", B3, "','", C3, "','", D3, "');")</f>
-        <v>INSERT INTO supplier (id, name, phone, email) values (2,'Thiri Mon','09-1122-2234','aunggabar@example.com');</v>
+        <v>INSERT INTO supplier (id, name, phone, email) values (2,'Thiri Mon','09-1122-2234','thiri@example.com');</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -875,11 +884,11 @@
         <v>37</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>32</v>
+        <v>61</v>
       </c>
       <c r="E4" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO supplier (id, name, phone, email) values (3,'Nyein Myitter','09-1122-2235','aunggabar@example.com');</v>
+        <v>INSERT INTO supplier (id, name, phone, email) values (3,'Nyein Myitter','09-1122-2235','nyein@example.com');</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -893,11 +902,11 @@
         <v>38</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>32</v>
+        <v>62</v>
       </c>
       <c r="E5" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO supplier (id, name, phone, email) values (4,'Shwe Store','09-1122-2236','aunggabar@example.com');</v>
+        <v>INSERT INTO supplier (id, name, phone, email) values (4,'Shwe Store','09-1122-2236','shwe@example.com');</v>
       </c>
     </row>
   </sheetData>
@@ -937,8 +946,8 @@
         <v>39</v>
       </c>
       <c r="C2" t="str">
-        <f>_xlfn.CONCAT("INSERT INTO PRODUCT (", A$1, ", ",B$1, ") values (", A2, ",'", B2, "');")</f>
-        <v>INSERT INTO PRODUCT (id, name) values (1,'Coke');</v>
+        <f>_xlfn.CONCAT("INSERT INTO product (", A$1, ", ",B$1, ") values (", A2, ",'", B2, "');")</f>
+        <v>INSERT INTO product (id, name) values (1,'Coke');</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -949,8 +958,8 @@
         <v>40</v>
       </c>
       <c r="C3" t="str">
-        <f>_xlfn.CONCAT("INSERT INTO PRODUCT (", A$1, ", ",B$1, ") values (", A3, ",'", B3, "');")</f>
-        <v>INSERT INTO PRODUCT (id, name) values (2,'Pepsi');</v>
+        <f t="shared" ref="C3:C4" si="0">_xlfn.CONCAT("INSERT INTO product (", A$1, ", ",B$1, ") values (", A3, ",'", B3, "');")</f>
+        <v>INSERT INTO product (id, name) values (2,'Pepsi');</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -961,8 +970,8 @@
         <v>41</v>
       </c>
       <c r="C4" t="str">
-        <f>_xlfn.CONCAT("INSERT INTO PRODUCT (", A$1, ", ",B$1, ") values (", A4, ",'", B4, "');")</f>
-        <v>INSERT INTO PRODUCT (id, name) values (3,'Nest Café');</v>
+        <f t="shared" si="0"/>
+        <v>INSERT INTO product (id, name) values (3,'Nest Café');</v>
       </c>
     </row>
   </sheetData>
@@ -1015,8 +1024,8 @@
         <v>0</v>
       </c>
       <c r="F2" t="str">
-        <f>_xlfn.CONCAT("INSERT INTO STOCK (", A$1, ", ",B$1, ", ", C$1, ", ",D$1, ", ",E$1, ") values (", A2, ",", B2, ",", C2, ",", D2, ",", E2, ");")</f>
-        <v>INSERT INTO STOCK (product_id, version, stock_amount, purchase_price, sale_price) values (1,0,0,0,0);</v>
+        <f>_xlfn.CONCAT("INSERT INTO stock (", A$1, ", ",B$1, ", ", C$1, ", ",D$1, ", ",E$1, ") values (", A2, ",", B2, ",", C2, ",", D2, ",", E2, ");")</f>
+        <v>INSERT INTO stock (product_id, version, stock_amount, purchase_price, sale_price) values (1,0,0,0,0);</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -1037,8 +1046,8 @@
         <v>2200</v>
       </c>
       <c r="F3" t="str">
-        <f>_xlfn.CONCAT("INSERT INTO STOCK (", A$1, ", ",B$1, ", ", C$1, ", ",D$1, ", ",E$1, ") values (", A3, ",", B3, ",", C3, ",", D3, ",", E3, ");")</f>
-        <v>INSERT INTO STOCK (product_id, version, stock_amount, purchase_price, sale_price) values (2,1,100,2000,2200);</v>
+        <f t="shared" ref="F3:F4" si="0">_xlfn.CONCAT("INSERT INTO stock (", A$1, ", ",B$1, ", ", C$1, ", ",D$1, ", ",E$1, ") values (", A3, ",", B3, ",", C3, ",", D3, ",", E3, ");")</f>
+        <v>INSERT INTO stock (product_id, version, stock_amount, purchase_price, sale_price) values (2,1,100,2000,2200);</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -1059,8 +1068,8 @@
         <v>3300</v>
       </c>
       <c r="F4" t="str">
-        <f>_xlfn.CONCAT("INSERT INTO STOCK (", A$1, ", ",B$1, ", ", C$1, ", ",D$1, ", ",E$1, ") values (", A4, ",", B4, ",", C4, ",", D4, ",", E4, ");")</f>
-        <v>INSERT INTO STOCK (product_id, version, stock_amount, purchase_price, sale_price) values (3,1,100,3000,3300);</v>
+        <f t="shared" si="0"/>
+        <v>INSERT INTO stock (product_id, version, stock_amount, purchase_price, sale_price) values (3,1,100,3000,3300);</v>
       </c>
     </row>
   </sheetData>
@@ -1118,8 +1127,8 @@
         <v>0</v>
       </c>
       <c r="G2" t="str">
-        <f>_xlfn.CONCAT("INSERT INTO STOCK_HISTORY (", A$1, ", ",B$1, ", ", C$1, ", ",D$1, ", ",E$1, ", ",F$1, ") values (", A2, ",", B2, ",'", C2, "' ,", D2, ",", E2, ",", F2, ");")</f>
-        <v>INSERT INTO STOCK_HISTORY (product_id, version, action_type, purchase_price, sale_price, amount) values (1,0,'Initiate' ,0,0,0);</v>
+        <f>_xlfn.CONCAT("INSERT INTO stock_history (", A$1, ", ",B$1, ", ", C$1, ", ",D$1, ", ",E$1, ", ",F$1, ") values (", A2, ",", B2, ",'", C2, "' ,", D2, ",", E2, ",", F2, ");")</f>
+        <v>INSERT INTO stock_history (product_id, version, action_type, purchase_price, sale_price, amount) values (1,0,'Initiate' ,0,0,0);</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -1142,8 +1151,8 @@
         <v>0</v>
       </c>
       <c r="G3" t="str">
-        <f t="shared" ref="G3:G6" si="0">_xlfn.CONCAT("INSERT INTO STOCK_HISTORY (", A$1, ", ",B$1, ", ", C$1, ", ",D$1, ", ",E$1, ", ",F$1, ") values (", A3, ",", B3, ",'", C3, "' ,", D3, ",", E3, ",", F3, ");")</f>
-        <v>INSERT INTO STOCK_HISTORY (product_id, version, action_type, purchase_price, sale_price, amount) values (2,0,'Initiate' ,0,0,0);</v>
+        <f t="shared" ref="G3:G6" si="0">_xlfn.CONCAT("INSERT INTO stock_history (", A$1, ", ",B$1, ", ", C$1, ", ",D$1, ", ",E$1, ", ",F$1, ") values (", A3, ",", B3, ",'", C3, "' ,", D3, ",", E3, ",", F3, ");")</f>
+        <v>INSERT INTO stock_history (product_id, version, action_type, purchase_price, sale_price, amount) values (2,0,'Initiate' ,0,0,0);</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -1167,7 +1176,7 @@
       </c>
       <c r="G4" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO STOCK_HISTORY (product_id, version, action_type, purchase_price, sale_price, amount) values (3,0,'Initiate' ,0,0,0);</v>
+        <v>INSERT INTO stock_history (product_id, version, action_type, purchase_price, sale_price, amount) values (3,0,'Initiate' ,0,0,0);</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -1192,7 +1201,7 @@
       </c>
       <c r="G5" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO STOCK_HISTORY (product_id, version, action_type, purchase_price, sale_price, amount) values (2,1,'Purchase' ,2000,2200,100);</v>
+        <v>INSERT INTO stock_history (product_id, version, action_type, purchase_price, sale_price, amount) values (2,1,'Purchase' ,2000,2200,100);</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -1217,7 +1226,7 @@
       </c>
       <c r="G6" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO STOCK_HISTORY (product_id, version, action_type, purchase_price, sale_price, amount) values (3,1,'Purchase' ,3000,3300,100);</v>
+        <v>INSERT INTO stock_history (product_id, version, action_type, purchase_price, sale_price, amount) values (3,1,'Purchase' ,3000,3300,100);</v>
       </c>
     </row>
   </sheetData>
@@ -1250,8 +1259,8 @@
         <v>1</v>
       </c>
       <c r="C2" t="str">
-        <f>_xlfn.CONCAT("INSERT INTO PRODUCT_SUPPLIER (", A$1, ", ",B$1, ") values (", A2, ",", B2, ");")</f>
-        <v>INSERT INTO PRODUCT_SUPPLIER (product_id, supplier_id) values (1,1);</v>
+        <f>_xlfn.CONCAT("INSERT INTO product_supplier (", A$1, ", ",B$1, ") values (", A2, ",", B2, ");")</f>
+        <v>INSERT INTO product_supplier (product_id, supplier_id) values (1,1);</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -1262,8 +1271,8 @@
         <v>1</v>
       </c>
       <c r="C3" t="str">
-        <f>_xlfn.CONCAT("INSERT INTO PRODUCT_SUPPLIER (", A$1, ", ",B$1, ") values (", A3, ",", B3, ");")</f>
-        <v>INSERT INTO PRODUCT_SUPPLIER (product_id, supplier_id) values (2,1);</v>
+        <f t="shared" ref="C3:C4" si="0">_xlfn.CONCAT("INSERT INTO product_supplier (", A$1, ", ",B$1, ") values (", A3, ",", B3, ");")</f>
+        <v>INSERT INTO product_supplier (product_id, supplier_id) values (2,1);</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -1274,8 +1283,8 @@
         <v>1</v>
       </c>
       <c r="C4" t="str">
-        <f>_xlfn.CONCAT("INSERT INTO PRODUCT_SUPPLIER (", A$1, ", ",B$1, ") values (", A4, ",", B4, ");")</f>
-        <v>INSERT INTO PRODUCT_SUPPLIER (product_id, supplier_id) values (3,1);</v>
+        <f t="shared" si="0"/>
+        <v>INSERT INTO product_supplier (product_id, supplier_id) values (3,1);</v>
       </c>
     </row>
   </sheetData>
@@ -1327,8 +1336,8 @@
         <v>15000</v>
       </c>
       <c r="F2" t="str">
-        <f>_xlfn.CONCAT("INSERT INTO PRUCHASE (", A$1, ", ",B$1, ", ", C$1, ", ",D$1, ", ",E$1, ") values (", A2, ",", B2, ",", C2, ",'", D2, "' ,", E2, ");")</f>
-        <v>INSERT INTO PRUCHASE (id, employee_id, supplier_id, purchase_date, transportation_fee) values (1,1,1,'2026-04-10' ,15000);</v>
+        <f>_xlfn.CONCAT("INSERT INTO purchase (", A$1, ", ",B$1, ", ", C$1, ", ",D$1, ", ",E$1, ") values (", A2, ",", B2, ",", C2, ",'", D2, "' ,", E2, ");")</f>
+        <v>INSERT INTO purchase (id, employee_id, supplier_id, purchase_date, transportation_fee) values (1,1,1,'2026-04-10' ,15000);</v>
       </c>
     </row>
   </sheetData>
@@ -1375,8 +1384,8 @@
         <v>100</v>
       </c>
       <c r="F2" t="str">
-        <f>_xlfn.CONCAT("INSERT INTO PRUCHASE_PRODUCT (", A$1, ", ",B$1, ", ", C$1, ", ",D$1, ", ",E$1, ") values (", A2, ",", B2, ",", C2, ",", D2, ",", E2, ");")</f>
-        <v>INSERT INTO PRUCHASE_PRODUCT (product_id, version, purchase_id, unit_price, quantity) values (2,1,1,2000,100);</v>
+        <f>_xlfn.CONCAT("INSERT INTO purchase_product (", A$1, ", ",B$1, ", ", C$1, ", ",D$1, ", ",E$1, ") values (", A2, ",", B2, ",", C2, ",", D2, ",", E2, ");")</f>
+        <v>INSERT INTO purchase_product (product_id, version, purchase_id, unit_price, quantity) values (2,1,1,2000,100);</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -1396,8 +1405,8 @@
         <v>100</v>
       </c>
       <c r="F3" t="str">
-        <f>_xlfn.CONCAT("INSERT INTO PRUCHASE_PRODUCT (", A$1, ", ",B$1, ", ", C$1, ", ",D$1, ", ",E$1, ") values (", A3, ",", B3, ",", C3, ",", D3, ",", E3, ");")</f>
-        <v>INSERT INTO PRUCHASE_PRODUCT (product_id, version, purchase_id, unit_price, quantity) values (3,1,1,3000,100);</v>
+        <f>_xlfn.CONCAT("INSERT INTO purchase_product (", A$1, ", ",B$1, ", ", C$1, ", ",D$1, ", ",E$1, ") values (", A3, ",", B3, ",", C3, ",", D3, ",", E3, ");")</f>
+        <v>INSERT INTO purchase_product (product_id, version, purchase_id, unit_price, quantity) values (3,1,1,3000,100);</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Test Cases for Transaction Management
</commit_message>
<xml_diff>
--- a/ep16-spring-transaction/online-shop-test-data.xlsx
+++ b/ep16-spring-transaction/online-shop-test-data.xlsx
@@ -8,22 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/minlwin/git/spring-weekend-202603/ep16-spring-transaction/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38AA209C-EBCC-2849-A123-BA5EFA83BDD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{774B7965-B773-674E-BCE3-19BFE4E9E075}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2320" yWindow="660" windowWidth="25600" windowHeight="12800" xr2:uid="{B0DF375E-B9E1-2C42-A1BE-A72AC035EBB6}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" activeTab="5" xr2:uid="{B0DF375E-B9E1-2C42-A1BE-A72AC035EBB6}"/>
   </bookViews>
   <sheets>
     <sheet name="CRUD" sheetId="5" r:id="rId1"/>
     <sheet name="EMPLOYEE" sheetId="1" r:id="rId2"/>
     <sheet name="SUPPLIER" sheetId="2" r:id="rId3"/>
-    <sheet name="PRODUCT" sheetId="3" r:id="rId4"/>
-    <sheet name="STOCK" sheetId="4" r:id="rId5"/>
-    <sheet name="STOCK_HISTORY" sheetId="7" r:id="rId6"/>
-    <sheet name="PRODUCT_SUPPLIER" sheetId="6" r:id="rId7"/>
-    <sheet name="PURCHASE" sheetId="8" r:id="rId8"/>
-    <sheet name="PURCHASE_PRODUCT" sheetId="9" r:id="rId9"/>
+    <sheet name="CUSTOMER" sheetId="10" r:id="rId4"/>
+    <sheet name="PRODUCT" sheetId="3" r:id="rId5"/>
+    <sheet name="STOCK" sheetId="4" r:id="rId6"/>
+    <sheet name="STOCK_HISTORY" sheetId="7" r:id="rId7"/>
+    <sheet name="PRODUCT_SUPPLIER" sheetId="6" r:id="rId8"/>
+    <sheet name="PURCHASE" sheetId="8" r:id="rId9"/>
+    <sheet name="PURCHASE_PRODUCT" sheetId="9" r:id="rId10"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="70">
   <si>
     <t>SUPPLIER</t>
   </si>
@@ -233,6 +234,27 @@
   </si>
   <si>
     <t>shwe@example.com</t>
+  </si>
+  <si>
+    <t>CUSTOMER</t>
+  </si>
+  <si>
+    <t>09-9122-2233</t>
+  </si>
+  <si>
+    <t>09-9122-2234</t>
+  </si>
+  <si>
+    <t>Min Aung</t>
+  </si>
+  <si>
+    <t>Htin Aung</t>
+  </si>
+  <si>
+    <t>minaung@example.com</t>
+  </si>
+  <si>
+    <t>htinaung@example.com</t>
   </si>
 </sst>
 </file>
@@ -264,7 +286,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -272,24 +294,46 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment textRotation="180"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" textRotation="180"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -625,108 +669,234 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7A75D78-218C-5245-B45D-86B7D30206F8}">
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.83203125" customWidth="1"/>
-    <col min="2" max="11" width="6.33203125" style="3" customWidth="1"/>
+    <col min="2" max="12" width="6.33203125" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" ht="116" x14ac:dyDescent="0.2">
-      <c r="B1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="2" t="s">
+    <row r="1" spans="1:12" s="1" customFormat="1" ht="116" x14ac:dyDescent="0.2">
+      <c r="A1" s="5"/>
+      <c r="B1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A2" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E2" s="3" t="s">
+      <c r="B2" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="I2" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="J2" s="8" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A3" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="B3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" s="8"/>
+      <c r="I3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="K3" s="8"/>
+      <c r="L3" s="8"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A4" s="7" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="B4" s="8"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4" s="8"/>
+      <c r="I4" s="8"/>
+      <c r="J4" s="8"/>
+      <c r="K4" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A5" s="7" t="s">
         <v>13</v>
+      </c>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" s="8"/>
+      <c r="I5" s="8"/>
+      <c r="J5" s="8"/>
+      <c r="K5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="L5" s="8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18B6CE9E-DE44-E245-9AB7-92515F40D1EA}">
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>2</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>2000</v>
+      </c>
+      <c r="E2">
+        <v>100</v>
+      </c>
+      <c r="F2" t="str">
+        <f>_xlfn.CONCAT("INSERT INTO purchase_product (", A$1, ", ",B$1, ", ", C$1, ", ",D$1, ", ",E$1, ") values (", A2, ",", B2, ",", C2, ",", D2, ",", E2, ");")</f>
+        <v>INSERT INTO purchase_product (product_id, version, purchase_id, unit_price, quantity) values (2,1,1,2000,100);</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>3000</v>
+      </c>
+      <c r="E3">
+        <v>100</v>
+      </c>
+      <c r="F3" t="str">
+        <f>_xlfn.CONCAT("INSERT INTO purchase_product (", A$1, ", ",B$1, ", ", C$1, ", ",D$1, ", ",E$1, ") values (", A3, ",", B3, ",", C3, ",", D3, ",", E3, ");")</f>
+        <v>INSERT INTO purchase_product (product_id, version, purchase_id, unit_price, quantity) values (3,1,1,3000,100);</v>
       </c>
     </row>
   </sheetData>
@@ -774,7 +944,7 @@
       <c r="D2" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>25</v>
       </c>
       <c r="F2" t="str">
@@ -795,7 +965,7 @@
       <c r="D3" t="s">
         <v>28</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F3" t="str">
@@ -847,7 +1017,7 @@
       <c r="C2" t="s">
         <v>31</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>32</v>
       </c>
       <c r="E2" t="str">
@@ -865,7 +1035,7 @@
       <c r="C3" t="s">
         <v>36</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="3" t="s">
         <v>60</v>
       </c>
       <c r="E3" t="str">
@@ -883,7 +1053,7 @@
       <c r="C4" t="s">
         <v>37</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E4" t="str">
@@ -901,7 +1071,7 @@
       <c r="C5" t="s">
         <v>38</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="3" t="s">
         <v>62</v>
       </c>
       <c r="E5" t="str">
@@ -921,6 +1091,74 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{523D8301-E88B-4841-93BF-7FF32466FFDF}">
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E2" t="str">
+        <f>_xlfn.CONCAT("INSERT INTO customer (", A$1, ", ",B$1, ", ",C$1, ", ",D$1, ") values (", A2, ",'", B2, "','", C2, "','", D2, "');")</f>
+        <v>INSERT INTO customer (id, name, phone, email) values (1,'Min Aung','09-9122-2233','minaung@example.com');</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C3" t="s">
+        <v>65</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E3" t="str">
+        <f>_xlfn.CONCAT("INSERT INTO customer (", A$1, ", ",B$1, ", ",C$1, ", ",D$1, ") values (", A3, ",'", B3, "','", C3, "','", D3, "');")</f>
+        <v>INSERT INTO customer (id, name, phone, email) values (2,'Htin Aung','09-9122-2234','htinaung@example.com');</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{4CCEBD61-D36B-914B-9439-A0BCD355AF2E}"/>
+    <hyperlink ref="D3" r:id="rId2" xr:uid="{15CBDC0E-A0AF-B545-A6C7-6CCEC27CD966}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A281D4A2-8D04-4D41-BC8D-CD3B12F93F5A}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -979,7 +1217,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2208E2B1-296B-934F-BAB6-3B2E64293929}">
   <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1077,7 +1315,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB877F23-7DA6-4C42-A722-09CE575D7EDD}">
   <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1234,7 +1472,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFB4A40D-58BB-704F-8F47-0B4C4C24FB0E}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1292,13 +1530,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFAC4344-ACE6-E245-9032-73EF7DF4D31F}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="13" customWidth="1"/>
-    <col min="4" max="4" width="20.33203125" style="5" customWidth="1"/>
+    <col min="4" max="4" width="20.33203125" style="4" customWidth="1"/>
     <col min="5" max="5" width="21.1640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1312,7 +1550,7 @@
       <c r="C1" t="s">
         <v>52</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>54</v>
       </c>
       <c r="E1" t="s">
@@ -1329,7 +1567,7 @@
       <c r="C2">
         <v>1</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="4" t="s">
         <v>56</v>
       </c>
       <c r="E2">
@@ -1338,75 +1576,6 @@
       <c r="F2" t="str">
         <f>_xlfn.CONCAT("INSERT INTO purchase (", A$1, ", ",B$1, ", ", C$1, ", ",D$1, ", ",E$1, ") values (", A2, ",", B2, ",", C2, ",'", D2, "' ,", E2, ");")</f>
         <v>INSERT INTO purchase (id, employee_id, supplier_id, purchase_date, transportation_fee) values (1,1,1,'2026-04-10' ,15000);</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18B6CE9E-DE44-E245-9AB7-92515F40D1EA}">
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D1" t="s">
-        <v>58</v>
-      </c>
-      <c r="E1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2">
-        <v>2</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>2000</v>
-      </c>
-      <c r="E2">
-        <v>100</v>
-      </c>
-      <c r="F2" t="str">
-        <f>_xlfn.CONCAT("INSERT INTO purchase_product (", A$1, ", ",B$1, ", ", C$1, ", ",D$1, ", ",E$1, ") values (", A2, ",", B2, ",", C2, ",", D2, ",", E2, ");")</f>
-        <v>INSERT INTO purchase_product (product_id, version, purchase_id, unit_price, quantity) values (2,1,1,2000,100);</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3">
-        <v>3</v>
-      </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>3000</v>
-      </c>
-      <c r="E3">
-        <v>100</v>
-      </c>
-      <c r="F3" t="str">
-        <f>_xlfn.CONCAT("INSERT INTO purchase_product (", A$1, ", ",B$1, ", ", C$1, ", ",D$1, ", ",E$1, ") values (", A3, ",", B3, ",", C3, ",", D3, ",", E3, ");")</f>
-        <v>INSERT INTO purchase_product (product_id, version, purchase_id, unit_price, quantity) values (3,1,1,3000,100);</v>
       </c>
     </row>
   </sheetData>

</xml_diff>